<commit_message>
Give the ThisWorkbook paste its own setup step
It was the tail of step 2, appended to "import every supplied .bas", so it
read as part of the import and got skipped. Pasting into a document class
module is a different action from importing a standard module, and it is the
only step in the sequence that cannot be done by File > Import. It is now its
own numbered step saying so, and saying what is lost by skipping it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_v0.2/python-annotator/excel-workbench/Entity-Gold-Review-Macro-Free.xlsx
+++ b/project_v0.2/python-annotator/excel-workbench/Entity-Gold-Review-Macro-Free.xlsx
@@ -19023,7 +19023,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Alt+F11 &gt; File &gt; Import File: import every supplied .bas. Paste ThisWorkbook.txt into the ThisWorkbook code window.</t>
+          <t>Alt+F11 &gt; File &gt; Import File: import all eight supplied .bas modules.</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
@@ -19043,7 +19043,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Alt+F8 &gt; SetupWorkbench &gt; Run creates the buttons. No manual shape wiring.</t>
+          <t>Separately, double-click ThisWorkbook under Microsoft Excel Objects and paste the whole of ThisWorkbook.txt into its empty code pane. This file cannot be imported, only pasted. Skipping it leaves the workbook without its reopen and close guards.</t>
         </is>
       </c>
       <c r="D6" s="1" t="n"/>
@@ -19063,7 +19063,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Notes: enter IDs, copy the full note, then Paste whole note. Or import UTF-8 TXT files named CLAIM_NOTE.txt.</t>
+          <t>Alt+F8 &gt; SetupWorkbench &gt; Run creates the buttons. No manual shape wiring.</t>
         </is>
       </c>
       <c r="D7" s="1" t="n"/>
@@ -19083,7 +19083,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Review Desk: choose entry kind, paste exact evidence, select occurrence and fill relevant fields. Choose entity lists accepted entities.</t>
+          <t>Notes: enter IDs, copy the full note, then Paste whole note. Or import UTF-8 TXT files named CLAIM_NOTE.txt.</t>
         </is>
       </c>
       <c r="D8" s="1" t="n"/>
@@ -19103,7 +19103,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Attest &amp; Save validates and saves. Save draft preserves unfinished work. Manual entry needs no Copilot.</t>
+          <t>Review Desk: choose entry kind, paste exact evidence, select occurrence and fill relevant fields. Choose entity lists accepted entities.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Optional AI: follow AI Instructions. SaveQueueSnapshot validates drafts, then Load next AI draft fills the form.</t>
+          <t>Attest &amp; Save validates and saves. Save draft preserves unfinished work. Manual entry needs no Copilot.</t>
         </is>
       </c>
       <c r="D10" s="1" t="n"/>
@@ -19143,7 +19143,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Previous entry restores your latest revision. Changed entries require new attestations; Delete preserves history.</t>
+          <t>Optional AI: follow AI Instructions. SaveQueueSnapshot validates drafts, then Load next AI draft fills the form.</t>
         </is>
       </c>
       <c r="D11" s="1" t="n"/>
@@ -19163,7 +19163,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Complete note requires reading all text, adding missing annotations and resolving drafts. Watchlist review follows.</t>
+          <t>Previous entry restores your latest revision. Changed entries require new attestations; Delete preserves history.</t>
         </is>
       </c>
       <c r="D12" s="1" t="n"/>
@@ -19183,7 +19183,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Only analysis for the last five distinct notes pasted is retained. Sources, pending queues and accepted records persist.</t>
+          <t>Complete note requires reading all text, adding missing annotations and resolving drafts. Watchlist review follows.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -19203,7 +19203,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>One SME writer per workbook. Do not edit with Copilot while macros save. Do not edit backend tables.</t>
+          <t>Only analysis for the last five distinct notes pasted is retained. Sources, pending queues and accepted records persist.</t>
         </is>
       </c>
       <c r="D14" s="1" t="n"/>
@@ -19223,7 +19223,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Keep older workbooks untouched. Read WIRE-UP-IN-EXCEL.md before bringing historical annotations into this layout.</t>
+          <t>One SME writer per workbook. Do not edit with Copilot while macros save. Do not edit backend tables.</t>
         </is>
       </c>
       <c r="D15" s="1" t="n"/>
@@ -19243,7 +19243,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Licensed Windows Excel runtime qualification is still required. Macros do not run in Excel for the web.</t>
+          <t>Keep older workbooks untouched. Read WIRE-UP-IN-EXCEL.md before bringing historical annotations into this layout.</t>
         </is>
       </c>
       <c r="D16" s="1" t="n"/>
@@ -19254,10 +19254,18 @@
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="1" t="n"/>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>14.</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Licensed Windows Excel runtime qualification is still required. Macros do not run in Excel for the web.</t>
+        </is>
+      </c>
       <c r="D17" s="1" t="n"/>
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="n"/>

</xml_diff>